<commit_message>
Fix font rendering on Streamlit Cloud with bundled TTF fonts and packages.txt
</commit_message>
<xml_diff>
--- a/sample_data/sample_students_with_errors.xlsx
+++ b/sample_data/sample_students_with_errors.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -488,7 +488,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">

</xml_diff>